<commit_message>
auto sync 2026-05-22 18:00:09
</commit_message>
<xml_diff>
--- a/[서버]_FAP_정기점검/templates/dr_mock_training_check_2026.xlsx
+++ b/[서버]_FAP_정기점검/templates/dr_mock_training_check_2026.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sgjan\AppData\Roaming\MobaXterm\slash\mx86_64b\RemoteFiles\1313484_6_79\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\akfen\Documents\이거\05 참여 프로젝트\08 신세계 I&amp;C (네트워크,서버) [유지보수] - 경기 김포시 태장로 779 [신세계아이앤씨 데이터센터]\02 서버\03 작업\DR점검\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1FE4927-FBB5-480D-B941-F498D536C633}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD161054-151B-4E90-A02F-3D98B7B50EDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35925" yWindow="2070" windowWidth="21330" windowHeight="12960" firstSheet="1" activeTab="2" xr2:uid="{5DB6A6EA-ACAF-404C-8255-11ACC19C1A85}"/>
+    <workbookView xWindow="29880" yWindow="-120" windowWidth="27840" windowHeight="16440" firstSheet="1" activeTab="2" xr2:uid="{5DB6A6EA-ACAF-404C-8255-11ACC19C1A85}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -647,29 +647,29 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1012,13 +1012,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BFBDA8A-A085-47FC-9A94-89833E63918C}">
   <dimension ref="A1:F16"/>
-  <sheetFormatPr defaultColWidth="16.59765625" defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="16.625" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="33.09765625" customWidth="1"/>
-    <col min="3" max="3" width="22.8984375" customWidth="1"/>
+    <col min="2" max="2" width="33.125" customWidth="1"/>
+    <col min="3" max="3" width="22.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
@@ -1038,7 +1038,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="18" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="12"/>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -1050,90 +1050,90 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="31.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="17" t="s">
+    <row r="3" spans="1:6" ht="31.15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="17" t="s">
+      <c r="C3" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="15">
+      <c r="D3" s="18">
         <v>45561</v>
       </c>
       <c r="E3" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="17" t="s">
+      <c r="F3" s="13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="18" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="18"/>
-      <c r="B4" s="18"/>
-      <c r="C4" s="18"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="14"/>
-      <c r="F4" s="18"/>
-    </row>
-    <row r="5" spans="1:6" ht="31.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="17" t="s">
+    <row r="4" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="14"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="14"/>
+    </row>
+    <row r="5" spans="1:6" ht="31.15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="13" t="s">
         <v>20</v>
       </c>
       <c r="C5" s="16"/>
-      <c r="D5" s="15">
+      <c r="D5" s="18">
         <v>45591</v>
       </c>
       <c r="E5" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="17" t="s">
+      <c r="F5" s="13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="18" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A6" s="18"/>
-      <c r="B6" s="18"/>
-      <c r="C6" s="14"/>
-      <c r="D6" s="14"/>
-      <c r="E6" s="14"/>
-      <c r="F6" s="18"/>
-    </row>
-    <row r="7" spans="1:6" ht="31.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="17" t="s">
+    <row r="6" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="14"/>
+      <c r="B6" s="14"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="14"/>
+    </row>
+    <row r="7" spans="1:6" ht="31.15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B7" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="15">
+      <c r="D7" s="18">
         <v>45638</v>
       </c>
       <c r="E7" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="17" t="s">
+      <c r="F7" s="13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="64.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A8" s="18"/>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="18"/>
-    </row>
-    <row r="9" spans="1:6" ht="31.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="17" t="s">
+    <row r="8" spans="1:6" ht="64.900000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="14"/>
+      <c r="B8" s="17"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="14"/>
+    </row>
+    <row r="9" spans="1:6" ht="31.15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="13" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="16" t="s">
@@ -1142,26 +1142,26 @@
       <c r="C9" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="15">
+      <c r="D9" s="18">
         <v>45708</v>
       </c>
       <c r="E9" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="F9" s="17" t="s">
+      <c r="F9" s="13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="18" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A10" s="18"/>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="18"/>
-    </row>
-    <row r="11" spans="1:6" ht="93.6" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="17" t="s">
+    <row r="10" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="14"/>
+      <c r="B10" s="17"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="14"/>
+    </row>
+    <row r="11" spans="1:6" ht="93.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="13" t="s">
         <v>18</v>
       </c>
       <c r="B11" s="16"/>
@@ -1170,70 +1170,52 @@
       <c r="E11" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="F11" s="17" t="s">
+      <c r="F11" s="13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A12" s="20"/>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="15"/>
       <c r="B12" s="19"/>
       <c r="C12" s="19"/>
       <c r="D12" s="19"/>
       <c r="E12" s="19"/>
-      <c r="F12" s="20"/>
-    </row>
-    <row r="13" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="20"/>
+      <c r="F12" s="15"/>
+    </row>
+    <row r="13" spans="1:6" ht="17.45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="15"/>
       <c r="B13" s="19"/>
       <c r="C13" s="19"/>
       <c r="D13" s="19"/>
       <c r="E13" s="19"/>
-      <c r="F13" s="20"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A14" s="20"/>
+      <c r="F13" s="15"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="15"/>
       <c r="B14" s="19"/>
       <c r="C14" s="19"/>
       <c r="D14" s="19"/>
       <c r="E14" s="19"/>
-      <c r="F14" s="20"/>
-    </row>
-    <row r="15" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="20"/>
+      <c r="F14" s="15"/>
+    </row>
+    <row r="15" spans="1:6" ht="17.45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="15"/>
       <c r="B15" s="19"/>
       <c r="C15" s="19"/>
       <c r="D15" s="19"/>
       <c r="E15" s="19"/>
-      <c r="F15" s="20"/>
-    </row>
-    <row r="16" spans="1:6" ht="18" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="18"/>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="18"/>
+      <c r="F15" s="15"/>
+    </row>
+    <row r="16" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="14"/>
+      <c r="B16" s="17"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A11:A16"/>
-    <mergeCell ref="F11:F16"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="B11:B16"/>
-    <mergeCell ref="C11:C16"/>
-    <mergeCell ref="D11:D16"/>
-    <mergeCell ref="E11:E16"/>
     <mergeCell ref="B7:B8"/>
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="D7:D8"/>
@@ -1250,6 +1232,24 @@
     <mergeCell ref="C5:C6"/>
     <mergeCell ref="D5:D6"/>
     <mergeCell ref="E5:E6"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="B11:B16"/>
+    <mergeCell ref="C11:C16"/>
+    <mergeCell ref="D11:D16"/>
+    <mergeCell ref="E11:E16"/>
+    <mergeCell ref="F11:F16"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A11:A16"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1259,20 +1259,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF239F09-F92A-4B54-8AD5-3D711A7BBEA2}">
   <dimension ref="B1:G39"/>
-  <sheetFormatPr defaultColWidth="37.5" defaultRowHeight="30.6" customHeight="1" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="37.5" defaultRowHeight="30.6" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.59765625" style="4" customWidth="1"/>
-    <col min="2" max="2" width="28.19921875" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.625" style="4" customWidth="1"/>
+    <col min="2" max="2" width="28.25" style="4" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="37.5" style="4"/>
     <col min="4" max="4" width="36.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.69921875" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.09765625" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.69921875" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.75" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.125" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.75" style="4" bestFit="1" customWidth="1"/>
     <col min="8" max="16384" width="37.5" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45"/>
-    <row r="2" spans="2:7" ht="30.6" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="2:7" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="11" t="s">
         <v>0</v>
       </c>
@@ -1292,7 +1292,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="2:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:7" ht="14.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="12"/>
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
@@ -1300,62 +1300,62 @@
       <c r="F3" s="12"/>
       <c r="G3" s="12"/>
     </row>
-    <row r="4" spans="2:7" ht="30.6" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B4" s="17" t="s">
+    <row r="4" spans="2:7" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="17" t="s">
+      <c r="D4" s="13" t="s">
         <v>19</v>
       </c>
       <c r="E4" s="21">
         <v>45561</v>
       </c>
-      <c r="F4" s="17" t="s">
+      <c r="F4" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="G4" s="17" t="s">
+      <c r="G4" s="13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="2:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B5" s="18"/>
-      <c r="C5" s="18"/>
-      <c r="D5" s="18"/>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18"/>
-    </row>
-    <row r="6" spans="2:7" ht="31.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B6" s="17" t="s">
+    <row r="5" spans="2:7" ht="14.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
+    </row>
+    <row r="6" spans="2:7" ht="31.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="17" t="s">
+      <c r="C6" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="D6" s="17"/>
+      <c r="D6" s="13"/>
       <c r="E6" s="21">
         <v>45591</v>
       </c>
-      <c r="F6" s="17" t="s">
+      <c r="F6" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="G6" s="17" t="s">
+      <c r="G6" s="13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="2:7" ht="30.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B7" s="18"/>
-      <c r="C7" s="18"/>
-      <c r="D7" s="18"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="18"/>
-    </row>
-    <row r="8" spans="2:7" ht="30.6" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B8" s="17" t="s">
+    <row r="7" spans="2:7" ht="30.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+    </row>
+    <row r="8" spans="2:7" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="13" t="s">
         <v>16</v>
       </c>
       <c r="C8" s="22" t="s">
@@ -1367,110 +1367,110 @@
       <c r="E8" s="21">
         <v>45638</v>
       </c>
-      <c r="F8" s="17" t="s">
+      <c r="F8" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="G8" s="17" t="s">
+      <c r="G8" s="13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="2:7" ht="53.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B9" s="18"/>
-      <c r="C9" s="18"/>
-      <c r="D9" s="18"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="18"/>
-    </row>
-    <row r="10" spans="2:7" ht="30.6" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B10" s="17" t="s">
+    <row r="9" spans="2:7" ht="53.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B9" s="14"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
+    </row>
+    <row r="10" spans="2:7" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="17" t="s">
+      <c r="C10" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="D10" s="17" t="s">
+      <c r="D10" s="13" t="s">
         <v>24</v>
       </c>
       <c r="E10" s="21">
         <v>45708</v>
       </c>
-      <c r="F10" s="17" t="s">
+      <c r="F10" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="G10" s="17" t="s">
+      <c r="G10" s="13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B11" s="18"/>
-      <c r="C11" s="18"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="18"/>
-      <c r="G11" s="18"/>
-    </row>
-    <row r="12" spans="2:7" ht="10.199999999999999" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B12" s="17" t="s">
+    <row r="11" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B11" s="14"/>
+      <c r="C11" s="14"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="14"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="14"/>
+    </row>
+    <row r="12" spans="2:7" ht="10.15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="17" t="s">
+      <c r="C12" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="D12" s="17" t="s">
+      <c r="D12" s="13" t="s">
         <v>29</v>
       </c>
       <c r="E12" s="21">
         <v>45743</v>
       </c>
-      <c r="F12" s="17" t="s">
+      <c r="F12" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="G12" s="17" t="s">
+      <c r="G12" s="13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="2:7" ht="10.199999999999999" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B13" s="20"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="20"/>
-      <c r="F13" s="20"/>
-      <c r="G13" s="20"/>
-    </row>
-    <row r="14" spans="2:7" ht="10.199999999999999" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B14" s="20"/>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="20"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="20"/>
-    </row>
-    <row r="15" spans="2:7" ht="10.199999999999999" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B15" s="20"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="20"/>
-      <c r="E15" s="20"/>
-      <c r="F15" s="20"/>
-      <c r="G15" s="20"/>
-    </row>
-    <row r="16" spans="2:7" ht="10.199999999999999" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B16" s="20"/>
-      <c r="C16" s="20"/>
-      <c r="D16" s="20"/>
-      <c r="E16" s="20"/>
-      <c r="F16" s="20"/>
-      <c r="G16" s="20"/>
-    </row>
-    <row r="17" spans="2:7" ht="10.199999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B17" s="20"/>
-      <c r="C17" s="20"/>
-      <c r="D17" s="20"/>
-      <c r="E17" s="20"/>
-      <c r="F17" s="20"/>
-      <c r="G17" s="20"/>
-    </row>
-    <row r="18" spans="2:7" ht="78.599999999999994" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:7" ht="10.15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="15"/>
+    </row>
+    <row r="14" spans="2:7" ht="10.15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="15"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="15"/>
+    </row>
+    <row r="15" spans="2:7" ht="10.15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="15"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="15"/>
+    </row>
+    <row r="16" spans="2:7" ht="10.15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="15"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+    </row>
+    <row r="17" spans="2:7" ht="10.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B17" s="15"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="15"/>
+    </row>
+    <row r="18" spans="2:7" ht="68.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B18" s="5" t="s">
         <v>30</v>
       </c>
@@ -1490,7 +1490,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="19" spans="2:7" ht="31.8" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="19" spans="2:7" ht="27.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B19" s="5" t="s">
         <v>35</v>
       </c>
@@ -1510,7 +1510,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B20" s="5" t="s">
         <v>41</v>
       </c>
@@ -1530,7 +1530,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B21" s="5" t="s">
         <v>42</v>
       </c>
@@ -1550,7 +1550,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="22" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B22" s="5" t="s">
         <v>38</v>
       </c>
@@ -1570,7 +1570,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="23" spans="2:7" ht="47.4" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:7" ht="41.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B23" s="5" t="s">
         <v>47</v>
       </c>
@@ -1590,7 +1590,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="24" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B24" s="5" t="s">
         <v>47</v>
       </c>
@@ -1610,7 +1610,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="25" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B25" s="3" t="s">
         <v>52</v>
       </c>
@@ -1628,7 +1628,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="26" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B26" s="3" t="s">
         <v>54</v>
       </c>
@@ -1646,7 +1646,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="27" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="27" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" s="3" t="s">
         <v>55</v>
       </c>
@@ -1664,7 +1664,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="28" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="28" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B28" s="6" t="s">
         <v>58</v>
       </c>
@@ -1682,7 +1682,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="29" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="29" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B29" s="3" t="s">
         <v>61</v>
       </c>
@@ -1702,7 +1702,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="30" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="30" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B30" s="3" t="s">
         <v>16</v>
       </c>
@@ -1722,7 +1722,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="31" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="31" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B31" s="3" t="s">
         <v>62</v>
       </c>
@@ -1740,7 +1740,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="32" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="32" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B32" s="3" t="s">
         <v>63</v>
       </c>
@@ -1758,7 +1758,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="33" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="33" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B33" s="3" t="s">
         <v>65</v>
       </c>
@@ -1776,7 +1776,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="34" spans="2:7" ht="63" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="34" spans="2:7" ht="54.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B34" s="3" t="s">
         <v>67</v>
       </c>
@@ -1796,7 +1796,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="35" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="35" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B35" s="3" t="s">
         <v>47</v>
       </c>
@@ -1816,7 +1816,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="36" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="36" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B36" s="3" t="s">
         <v>68</v>
       </c>
@@ -1836,7 +1836,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="37" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="37" spans="2:7" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B37" s="3" t="s">
         <v>76</v>
       </c>
@@ -1856,7 +1856,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="38" spans="2:7" ht="47.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="38" spans="2:7" ht="47.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B38" s="3" t="s">
         <v>79</v>
       </c>
@@ -1876,7 +1876,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="39" spans="2:7" ht="41.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="39" spans="2:7" ht="41.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B39" s="3" t="s">
         <v>80</v>
       </c>
@@ -1894,6 +1894,26 @@
     </row>
   </sheetData>
   <mergeCells count="36">
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="F6:F7"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="G8:G9"/>
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="G4:G5"/>
+    <mergeCell ref="G6:G7"/>
     <mergeCell ref="F2:F3"/>
     <mergeCell ref="G2:G3"/>
     <mergeCell ref="B12:B17"/>
@@ -1910,26 +1930,6 @@
     <mergeCell ref="G10:G11"/>
     <mergeCell ref="B8:B9"/>
     <mergeCell ref="C8:C9"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="E8:E9"/>
-    <mergeCell ref="F8:F9"/>
-    <mergeCell ref="G8:G9"/>
-    <mergeCell ref="F4:F5"/>
-    <mergeCell ref="G4:G5"/>
-    <mergeCell ref="G6:G7"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="E6:E7"/>
-    <mergeCell ref="F6:F7"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:E5"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1939,17 +1939,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A51507AB-5F46-4D71-8493-D29A752282BF}">
   <dimension ref="B1:G10"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="22.3984375" customWidth="1"/>
+    <col min="2" max="2" width="22.375" customWidth="1"/>
     <col min="3" max="3" width="24.5" customWidth="1"/>
-    <col min="4" max="4" width="36.69921875" customWidth="1"/>
-    <col min="5" max="5" width="13.59765625" customWidth="1"/>
-    <col min="6" max="7" width="12.09765625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="36.75" customWidth="1"/>
+    <col min="5" max="5" width="13.625" customWidth="1"/>
+    <col min="6" max="7" width="12.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" ht="18" thickBot="1" x14ac:dyDescent="0.45"/>
-    <row r="2" spans="2:7" x14ac:dyDescent="0.4">
+    <row r="1" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B2" s="11" t="s">
         <v>0</v>
       </c>
@@ -1969,7 +1969,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="3" spans="2:7" ht="18" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="12"/>
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
@@ -1977,7 +1977,7 @@
       <c r="F3" s="12"/>
       <c r="G3" s="12"/>
     </row>
-    <row r="4" spans="2:7" ht="35.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:7" ht="35.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
         <v>65</v>
       </c>
@@ -1995,7 +1995,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="5" spans="2:7" ht="74.400000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:7" ht="57" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B5" s="3" t="s">
         <v>67</v>
       </c>
@@ -2015,7 +2015,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="2:7" ht="35.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:7" ht="35.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
         <v>47</v>
       </c>
@@ -2035,7 +2035,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="2:7" ht="35.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:7" ht="35.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B7" s="3" t="s">
         <v>68</v>
       </c>
@@ -2055,7 +2055,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="2:7" ht="35.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:7" ht="35.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B8" s="3" t="s">
         <v>76</v>
       </c>
@@ -2075,7 +2075,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="9" spans="2:7" ht="59.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:7" ht="59.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B9" s="3" t="s">
         <v>79</v>
       </c>
@@ -2095,7 +2095,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="2:7" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:7" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" s="3" t="s">
         <v>80</v>
       </c>

</xml_diff>